<commit_message>
Porte les plages de moniteurs à cinquante entrées
La validation des colonnes « Moniteur remplacé » et « Moniteur
remplaçant » s'arrêtait à la vingtième entrée de l'onglet Listes, et le
récapitulatif aussi : les moniteurs ajoutés au-delà n'apparaissaient ni
dans les menus déroulants ni dans les totaux.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RsDkbcD3KwyPviDTcs72WZ
</commit_message>
<xml_diff>
--- a/Remplacements_2026-2027.xlsx
+++ b/Remplacements_2026-2027.xlsx
@@ -4228,7 +4228,7 @@
   </mergeCells>
   <dataValidations count="3">
     <dataValidation allowBlank="true" error="Choisissez un moniteur dans la liste. Pour en ajouter un, complétez l’onglet « Listes »." errorStyle="stop" errorTitle="Moniteur inconnu" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D6:E255" type="list">
-      <formula1>Listes!$A$2:$A$21</formula1>
+      <formula1>Listes!$A$2:$A$51</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Choisissez un motif dans la liste." errorStyle="stop" errorTitle="Motif inconnu" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F6:F255" type="list">
@@ -4368,7 +4368,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -4854,41 +4854,701 @@
         <v/>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="24" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="18" t="str">
+        <f aca="false">IF(Listes!A22="","",Listes!A22)</f>
+        <v/>
+      </c>
+      <c r="B26" s="19" t="str">
+        <f aca="false">IF($A26="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A26,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C26" s="19" t="str">
+        <f aca="false">IF($A26="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A26,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D26" s="20" t="str">
+        <f aca="false">IF($A26="","",SUMIF(Remplacements!$E$6:$E$255,$A26,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E26" s="20" t="str">
+        <f aca="false">IF($A26="","",SUMIF(Remplacements!$D$6:$D$255,$A26,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="21" t="str">
+        <f aca="false">IF(Listes!A23="","",Listes!A23)</f>
+        <v/>
+      </c>
+      <c r="B27" s="22" t="str">
+        <f aca="false">IF($A27="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A27,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C27" s="22" t="str">
+        <f aca="false">IF($A27="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A27,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D27" s="23" t="str">
+        <f aca="false">IF($A27="","",SUMIF(Remplacements!$E$6:$E$255,$A27,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E27" s="23" t="str">
+        <f aca="false">IF($A27="","",SUMIF(Remplacements!$D$6:$D$255,$A27,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="18" t="str">
+        <f aca="false">IF(Listes!A24="","",Listes!A24)</f>
+        <v/>
+      </c>
+      <c r="B28" s="19" t="str">
+        <f aca="false">IF($A28="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A28,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C28" s="19" t="str">
+        <f aca="false">IF($A28="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A28,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D28" s="20" t="str">
+        <f aca="false">IF($A28="","",SUMIF(Remplacements!$E$6:$E$255,$A28,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E28" s="20" t="str">
+        <f aca="false">IF($A28="","",SUMIF(Remplacements!$D$6:$D$255,$A28,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="21" t="str">
+        <f aca="false">IF(Listes!A25="","",Listes!A25)</f>
+        <v/>
+      </c>
+      <c r="B29" s="22" t="str">
+        <f aca="false">IF($A29="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A29,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C29" s="22" t="str">
+        <f aca="false">IF($A29="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A29,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D29" s="23" t="str">
+        <f aca="false">IF($A29="","",SUMIF(Remplacements!$E$6:$E$255,$A29,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E29" s="23" t="str">
+        <f aca="false">IF($A29="","",SUMIF(Remplacements!$D$6:$D$255,$A29,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="18" t="str">
+        <f aca="false">IF(Listes!A26="","",Listes!A26)</f>
+        <v/>
+      </c>
+      <c r="B30" s="19" t="str">
+        <f aca="false">IF($A30="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A30,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C30" s="19" t="str">
+        <f aca="false">IF($A30="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A30,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D30" s="20" t="str">
+        <f aca="false">IF($A30="","",SUMIF(Remplacements!$E$6:$E$255,$A30,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E30" s="20" t="str">
+        <f aca="false">IF($A30="","",SUMIF(Remplacements!$D$6:$D$255,$A30,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="21" t="str">
+        <f aca="false">IF(Listes!A27="","",Listes!A27)</f>
+        <v/>
+      </c>
+      <c r="B31" s="22" t="str">
+        <f aca="false">IF($A31="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A31,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C31" s="22" t="str">
+        <f aca="false">IF($A31="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A31,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D31" s="23" t="str">
+        <f aca="false">IF($A31="","",SUMIF(Remplacements!$E$6:$E$255,$A31,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E31" s="23" t="str">
+        <f aca="false">IF($A31="","",SUMIF(Remplacements!$D$6:$D$255,$A31,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="18" t="str">
+        <f aca="false">IF(Listes!A28="","",Listes!A28)</f>
+        <v/>
+      </c>
+      <c r="B32" s="19" t="str">
+        <f aca="false">IF($A32="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A32,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C32" s="19" t="str">
+        <f aca="false">IF($A32="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A32,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D32" s="20" t="str">
+        <f aca="false">IF($A32="","",SUMIF(Remplacements!$E$6:$E$255,$A32,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E32" s="20" t="str">
+        <f aca="false">IF($A32="","",SUMIF(Remplacements!$D$6:$D$255,$A32,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="21" t="str">
+        <f aca="false">IF(Listes!A29="","",Listes!A29)</f>
+        <v/>
+      </c>
+      <c r="B33" s="22" t="str">
+        <f aca="false">IF($A33="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A33,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C33" s="22" t="str">
+        <f aca="false">IF($A33="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A33,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D33" s="23" t="str">
+        <f aca="false">IF($A33="","",SUMIF(Remplacements!$E$6:$E$255,$A33,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E33" s="23" t="str">
+        <f aca="false">IF($A33="","",SUMIF(Remplacements!$D$6:$D$255,$A33,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="18" t="str">
+        <f aca="false">IF(Listes!A30="","",Listes!A30)</f>
+        <v/>
+      </c>
+      <c r="B34" s="19" t="str">
+        <f aca="false">IF($A34="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A34,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C34" s="19" t="str">
+        <f aca="false">IF($A34="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A34,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D34" s="20" t="str">
+        <f aca="false">IF($A34="","",SUMIF(Remplacements!$E$6:$E$255,$A34,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E34" s="20" t="str">
+        <f aca="false">IF($A34="","",SUMIF(Remplacements!$D$6:$D$255,$A34,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="21" t="str">
+        <f aca="false">IF(Listes!A31="","",Listes!A31)</f>
+        <v/>
+      </c>
+      <c r="B35" s="22" t="str">
+        <f aca="false">IF($A35="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A35,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C35" s="22" t="str">
+        <f aca="false">IF($A35="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A35,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D35" s="23" t="str">
+        <f aca="false">IF($A35="","",SUMIF(Remplacements!$E$6:$E$255,$A35,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E35" s="23" t="str">
+        <f aca="false">IF($A35="","",SUMIF(Remplacements!$D$6:$D$255,$A35,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="18" t="str">
+        <f aca="false">IF(Listes!A32="","",Listes!A32)</f>
+        <v/>
+      </c>
+      <c r="B36" s="19" t="str">
+        <f aca="false">IF($A36="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A36,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C36" s="19" t="str">
+        <f aca="false">IF($A36="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A36,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D36" s="20" t="str">
+        <f aca="false">IF($A36="","",SUMIF(Remplacements!$E$6:$E$255,$A36,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E36" s="20" t="str">
+        <f aca="false">IF($A36="","",SUMIF(Remplacements!$D$6:$D$255,$A36,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="21" t="str">
+        <f aca="false">IF(Listes!A33="","",Listes!A33)</f>
+        <v/>
+      </c>
+      <c r="B37" s="22" t="str">
+        <f aca="false">IF($A37="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A37,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C37" s="22" t="str">
+        <f aca="false">IF($A37="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A37,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D37" s="23" t="str">
+        <f aca="false">IF($A37="","",SUMIF(Remplacements!$E$6:$E$255,$A37,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E37" s="23" t="str">
+        <f aca="false">IF($A37="","",SUMIF(Remplacements!$D$6:$D$255,$A37,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="18" t="str">
+        <f aca="false">IF(Listes!A34="","",Listes!A34)</f>
+        <v/>
+      </c>
+      <c r="B38" s="19" t="str">
+        <f aca="false">IF($A38="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A38,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C38" s="19" t="str">
+        <f aca="false">IF($A38="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A38,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D38" s="20" t="str">
+        <f aca="false">IF($A38="","",SUMIF(Remplacements!$E$6:$E$255,$A38,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E38" s="20" t="str">
+        <f aca="false">IF($A38="","",SUMIF(Remplacements!$D$6:$D$255,$A38,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="21" t="str">
+        <f aca="false">IF(Listes!A35="","",Listes!A35)</f>
+        <v/>
+      </c>
+      <c r="B39" s="22" t="str">
+        <f aca="false">IF($A39="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A39,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C39" s="22" t="str">
+        <f aca="false">IF($A39="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A39,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D39" s="23" t="str">
+        <f aca="false">IF($A39="","",SUMIF(Remplacements!$E$6:$E$255,$A39,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E39" s="23" t="str">
+        <f aca="false">IF($A39="","",SUMIF(Remplacements!$D$6:$D$255,$A39,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="18" t="str">
+        <f aca="false">IF(Listes!A36="","",Listes!A36)</f>
+        <v/>
+      </c>
+      <c r="B40" s="19" t="str">
+        <f aca="false">IF($A40="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A40,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C40" s="19" t="str">
+        <f aca="false">IF($A40="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A40,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D40" s="20" t="str">
+        <f aca="false">IF($A40="","",SUMIF(Remplacements!$E$6:$E$255,$A40,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E40" s="20" t="str">
+        <f aca="false">IF($A40="","",SUMIF(Remplacements!$D$6:$D$255,$A40,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="21" t="str">
+        <f aca="false">IF(Listes!A37="","",Listes!A37)</f>
+        <v/>
+      </c>
+      <c r="B41" s="22" t="str">
+        <f aca="false">IF($A41="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A41,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C41" s="22" t="str">
+        <f aca="false">IF($A41="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A41,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D41" s="23" t="str">
+        <f aca="false">IF($A41="","",SUMIF(Remplacements!$E$6:$E$255,$A41,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E41" s="23" t="str">
+        <f aca="false">IF($A41="","",SUMIF(Remplacements!$D$6:$D$255,$A41,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="18" t="str">
+        <f aca="false">IF(Listes!A38="","",Listes!A38)</f>
+        <v/>
+      </c>
+      <c r="B42" s="19" t="str">
+        <f aca="false">IF($A42="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A42,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C42" s="19" t="str">
+        <f aca="false">IF($A42="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A42,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D42" s="20" t="str">
+        <f aca="false">IF($A42="","",SUMIF(Remplacements!$E$6:$E$255,$A42,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E42" s="20" t="str">
+        <f aca="false">IF($A42="","",SUMIF(Remplacements!$D$6:$D$255,$A42,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="21" t="str">
+        <f aca="false">IF(Listes!A39="","",Listes!A39)</f>
+        <v/>
+      </c>
+      <c r="B43" s="22" t="str">
+        <f aca="false">IF($A43="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A43,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C43" s="22" t="str">
+        <f aca="false">IF($A43="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A43,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D43" s="23" t="str">
+        <f aca="false">IF($A43="","",SUMIF(Remplacements!$E$6:$E$255,$A43,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E43" s="23" t="str">
+        <f aca="false">IF($A43="","",SUMIF(Remplacements!$D$6:$D$255,$A43,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="18" t="str">
+        <f aca="false">IF(Listes!A40="","",Listes!A40)</f>
+        <v/>
+      </c>
+      <c r="B44" s="19" t="str">
+        <f aca="false">IF($A44="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A44,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C44" s="19" t="str">
+        <f aca="false">IF($A44="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A44,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D44" s="20" t="str">
+        <f aca="false">IF($A44="","",SUMIF(Remplacements!$E$6:$E$255,$A44,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E44" s="20" t="str">
+        <f aca="false">IF($A44="","",SUMIF(Remplacements!$D$6:$D$255,$A44,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="21" t="str">
+        <f aca="false">IF(Listes!A41="","",Listes!A41)</f>
+        <v/>
+      </c>
+      <c r="B45" s="22" t="str">
+        <f aca="false">IF($A45="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A45,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C45" s="22" t="str">
+        <f aca="false">IF($A45="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A45,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D45" s="23" t="str">
+        <f aca="false">IF($A45="","",SUMIF(Remplacements!$E$6:$E$255,$A45,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E45" s="23" t="str">
+        <f aca="false">IF($A45="","",SUMIF(Remplacements!$D$6:$D$255,$A45,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="18" t="str">
+        <f aca="false">IF(Listes!A42="","",Listes!A42)</f>
+        <v/>
+      </c>
+      <c r="B46" s="19" t="str">
+        <f aca="false">IF($A46="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A46,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C46" s="19" t="str">
+        <f aca="false">IF($A46="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A46,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D46" s="20" t="str">
+        <f aca="false">IF($A46="","",SUMIF(Remplacements!$E$6:$E$255,$A46,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E46" s="20" t="str">
+        <f aca="false">IF($A46="","",SUMIF(Remplacements!$D$6:$D$255,$A46,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="21" t="str">
+        <f aca="false">IF(Listes!A43="","",Listes!A43)</f>
+        <v/>
+      </c>
+      <c r="B47" s="22" t="str">
+        <f aca="false">IF($A47="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A47,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C47" s="22" t="str">
+        <f aca="false">IF($A47="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A47,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D47" s="23" t="str">
+        <f aca="false">IF($A47="","",SUMIF(Remplacements!$E$6:$E$255,$A47,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E47" s="23" t="str">
+        <f aca="false">IF($A47="","",SUMIF(Remplacements!$D$6:$D$255,$A47,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="18" t="str">
+        <f aca="false">IF(Listes!A44="","",Listes!A44)</f>
+        <v/>
+      </c>
+      <c r="B48" s="19" t="str">
+        <f aca="false">IF($A48="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A48,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C48" s="19" t="str">
+        <f aca="false">IF($A48="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A48,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D48" s="20" t="str">
+        <f aca="false">IF($A48="","",SUMIF(Remplacements!$E$6:$E$255,$A48,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E48" s="20" t="str">
+        <f aca="false">IF($A48="","",SUMIF(Remplacements!$D$6:$D$255,$A48,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="21" t="str">
+        <f aca="false">IF(Listes!A45="","",Listes!A45)</f>
+        <v/>
+      </c>
+      <c r="B49" s="22" t="str">
+        <f aca="false">IF($A49="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A49,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C49" s="22" t="str">
+        <f aca="false">IF($A49="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A49,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D49" s="23" t="str">
+        <f aca="false">IF($A49="","",SUMIF(Remplacements!$E$6:$E$255,$A49,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E49" s="23" t="str">
+        <f aca="false">IF($A49="","",SUMIF(Remplacements!$D$6:$D$255,$A49,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="18" t="str">
+        <f aca="false">IF(Listes!A46="","",Listes!A46)</f>
+        <v/>
+      </c>
+      <c r="B50" s="19" t="str">
+        <f aca="false">IF($A50="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A50,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C50" s="19" t="str">
+        <f aca="false">IF($A50="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A50,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D50" s="20" t="str">
+        <f aca="false">IF($A50="","",SUMIF(Remplacements!$E$6:$E$255,$A50,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E50" s="20" t="str">
+        <f aca="false">IF($A50="","",SUMIF(Remplacements!$D$6:$D$255,$A50,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="21" t="str">
+        <f aca="false">IF(Listes!A47="","",Listes!A47)</f>
+        <v/>
+      </c>
+      <c r="B51" s="22" t="str">
+        <f aca="false">IF($A51="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A51,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C51" s="22" t="str">
+        <f aca="false">IF($A51="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A51,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D51" s="23" t="str">
+        <f aca="false">IF($A51="","",SUMIF(Remplacements!$E$6:$E$255,$A51,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E51" s="23" t="str">
+        <f aca="false">IF($A51="","",SUMIF(Remplacements!$D$6:$D$255,$A51,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="18" t="str">
+        <f aca="false">IF(Listes!A48="","",Listes!A48)</f>
+        <v/>
+      </c>
+      <c r="B52" s="19" t="str">
+        <f aca="false">IF($A52="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A52,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C52" s="19" t="str">
+        <f aca="false">IF($A52="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A52,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D52" s="20" t="str">
+        <f aca="false">IF($A52="","",SUMIF(Remplacements!$E$6:$E$255,$A52,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E52" s="20" t="str">
+        <f aca="false">IF($A52="","",SUMIF(Remplacements!$D$6:$D$255,$A52,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="21" t="str">
+        <f aca="false">IF(Listes!A49="","",Listes!A49)</f>
+        <v/>
+      </c>
+      <c r="B53" s="22" t="str">
+        <f aca="false">IF($A53="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A53,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C53" s="22" t="str">
+        <f aca="false">IF($A53="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A53,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D53" s="23" t="str">
+        <f aca="false">IF($A53="","",SUMIF(Remplacements!$E$6:$E$255,$A53,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E53" s="23" t="str">
+        <f aca="false">IF($A53="","",SUMIF(Remplacements!$D$6:$D$255,$A53,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="18" t="str">
+        <f aca="false">IF(Listes!A50="","",Listes!A50)</f>
+        <v/>
+      </c>
+      <c r="B54" s="19" t="str">
+        <f aca="false">IF($A54="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A54,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C54" s="19" t="str">
+        <f aca="false">IF($A54="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A54,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D54" s="20" t="str">
+        <f aca="false">IF($A54="","",SUMIF(Remplacements!$E$6:$E$255,$A54,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E54" s="20" t="str">
+        <f aca="false">IF($A54="","",SUMIF(Remplacements!$D$6:$D$255,$A54,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="21" t="str">
+        <f aca="false">IF(Listes!A51="","",Listes!A51)</f>
+        <v/>
+      </c>
+      <c r="B55" s="22" t="str">
+        <f aca="false">IF($A55="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A55,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="C55" s="22" t="str">
+        <f aca="false">IF($A55="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A55,Remplacements!$G$6:$G$255,$B$3))</f>
+        <v/>
+      </c>
+      <c r="D55" s="23" t="str">
+        <f aca="false">IF($A55="","",SUMIF(Remplacements!$E$6:$E$255,$A55,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+      <c r="E55" s="23" t="str">
+        <f aca="false">IF($A55="","",SUMIF(Remplacements!$D$6:$D$255,$A55,Remplacements!$C$6:$C$255))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="B27" s="25" t="n">
-        <f aca="false">SUM(B6:B25)</f>
+      <c r="B57" s="25" t="n">
+        <f aca="false">SUM(B6:B56)</f>
         <v>0</v>
       </c>
-      <c r="C27" s="25" t="n">
-        <f aca="false">SUM(C6:C25)</f>
+      <c r="C57" s="25" t="n">
+        <f aca="false">SUM(C6:C56)</f>
         <v>0</v>
       </c>
-      <c r="D27" s="25" t="n">
-        <f aca="false">SUM(D6:D25)</f>
+      <c r="D57" s="25" t="n">
+        <f aca="false">SUM(D6:D56)</f>
         <v>0</v>
       </c>
-      <c r="E27" s="25" t="n">
-        <f aca="false">SUM(E6:E25)</f>
+      <c r="E57" s="25" t="n">
+        <f aca="false">SUM(E6:E56)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="26" t="s">
+    <row r="59" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="B29" s="26"/>
-      <c r="C29" s="26"/>
-      <c r="D29" s="26"/>
-      <c r="E29" s="26"/>
+      <c r="B59" s="26"/>
+      <c r="C59" s="26"/>
+      <c r="D59" s="26"/>
+      <c r="E59" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="C3:E3"/>
-    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="A59:E59"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B3" type="list">
@@ -4911,7 +5571,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D55"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="1" style="0" width="18"/>
@@ -5099,23 +5759,203 @@
       <c r="C21" s="18"/>
       <c r="D21" s="18"/>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="26" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="28"/>
+      <c r="B22" s="18"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="18"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="28"/>
+      <c r="B23" s="18"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="18"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="28"/>
+      <c r="B24" s="18"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="28"/>
+      <c r="B25" s="18"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="28"/>
+      <c r="B26" s="18"/>
+      <c r="C26" s="18"/>
+      <c r="D26" s="18"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="28"/>
+      <c r="B27" s="18"/>
+      <c r="C27" s="18"/>
+      <c r="D27" s="18"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="28"/>
+      <c r="B28" s="18"/>
+      <c r="C28" s="18"/>
+      <c r="D28" s="18"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="28"/>
+      <c r="B29" s="18"/>
+      <c r="C29" s="18"/>
+      <c r="D29" s="18"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="28"/>
+      <c r="B30" s="18"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="18"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="28"/>
+      <c r="B31" s="18"/>
+      <c r="C31" s="18"/>
+      <c r="D31" s="18"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="28"/>
+      <c r="B32" s="18"/>
+      <c r="C32" s="18"/>
+      <c r="D32" s="18"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="28"/>
+      <c r="B33" s="18"/>
+      <c r="C33" s="18"/>
+      <c r="D33" s="18"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="28"/>
+      <c r="B34" s="18"/>
+      <c r="C34" s="18"/>
+      <c r="D34" s="18"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="28"/>
+      <c r="B35" s="18"/>
+      <c r="C35" s="18"/>
+      <c r="D35" s="18"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="28"/>
+      <c r="B36" s="18"/>
+      <c r="C36" s="18"/>
+      <c r="D36" s="18"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="28"/>
+      <c r="B37" s="18"/>
+      <c r="C37" s="18"/>
+      <c r="D37" s="18"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="28"/>
+      <c r="B38" s="18"/>
+      <c r="C38" s="18"/>
+      <c r="D38" s="18"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="28"/>
+      <c r="B39" s="18"/>
+      <c r="C39" s="18"/>
+      <c r="D39" s="18"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="28"/>
+      <c r="B40" s="18"/>
+      <c r="C40" s="18"/>
+      <c r="D40" s="18"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="28"/>
+      <c r="B41" s="18"/>
+      <c r="C41" s="18"/>
+      <c r="D41" s="18"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="28"/>
+      <c r="B42" s="18"/>
+      <c r="C42" s="18"/>
+      <c r="D42" s="18"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="28"/>
+      <c r="B43" s="18"/>
+      <c r="C43" s="18"/>
+      <c r="D43" s="18"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="28"/>
+      <c r="B44" s="18"/>
+      <c r="C44" s="18"/>
+      <c r="D44" s="18"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="28"/>
+      <c r="B45" s="18"/>
+      <c r="C45" s="18"/>
+      <c r="D45" s="18"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="28"/>
+      <c r="B46" s="18"/>
+      <c r="C46" s="18"/>
+      <c r="D46" s="18"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="28"/>
+      <c r="B47" s="18"/>
+      <c r="C47" s="18"/>
+      <c r="D47" s="18"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="28"/>
+      <c r="B48" s="18"/>
+      <c r="C48" s="18"/>
+      <c r="D48" s="18"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="28"/>
+      <c r="B49" s="18"/>
+      <c r="C49" s="18"/>
+      <c r="D49" s="18"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="28"/>
+      <c r="B50" s="18"/>
+      <c r="C50" s="18"/>
+      <c r="D50" s="18"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="28"/>
+      <c r="B51" s="18"/>
+      <c r="C51" s="18"/>
+      <c r="D51" s="18"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="B23" s="26"/>
-      <c r="C23" s="26"/>
-      <c r="D23" s="26"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="26"/>
-      <c r="B24" s="26"/>
-      <c r="C24" s="26"/>
-      <c r="D24" s="26"/>
+      <c r="B54" s="26"/>
+      <c r="C54" s="26"/>
+      <c r="D54" s="26"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="26"/>
+      <c r="B55" s="26"/>
+      <c r="C55" s="26"/>
+      <c r="D55" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A23:D24"/>
+    <mergeCell ref="A54:D55"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.4" right="0.4" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Reprend les vingt-trois moniteurs de la saison dans le fichier partagé
Les noms encodés en ligne sont repris dans l'onglet Listes, et les
plages étendues couvrent désormais les menus déroulants comme le
récapitulatif.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RsDkbcD3KwyPviDTcs72WZ
</commit_message>
<xml_diff>
--- a/Remplacements_2026-2027.xlsx
+++ b/Remplacements_2026-2027.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="84">
   <si>
     <t xml:space="preserve">REMPLACEMENTS — Saison 2026-2027</t>
   </si>
@@ -209,22 +209,76 @@
     <t xml:space="preserve">Mai</t>
   </si>
   <si>
+    <t xml:space="preserve">Thibault</t>
+  </si>
+  <si>
     <t xml:space="preserve">Juin</t>
   </si>
   <si>
+    <t xml:space="preserve">Philippe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Juillet</t>
   </si>
   <si>
+    <t xml:space="preserve">Adel</t>
+  </si>
+  <si>
     <t xml:space="preserve">Août</t>
   </si>
   <si>
+    <t xml:space="preserve">Alpaslan</t>
+  </si>
+  <si>
     <t xml:space="preserve">Septembre</t>
   </si>
   <si>
+    <t xml:space="preserve">Armelle</t>
+  </si>
+  <si>
     <t xml:space="preserve">Octobre</t>
   </si>
   <si>
+    <t xml:space="preserve">Celia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clément</t>
+  </si>
+  <si>
     <t xml:space="preserve">Décembre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fred</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guillaume</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jérémie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loïc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Morad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pascal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thibaut</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Xavier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zeliha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Camelia</t>
   </si>
   <si>
     <t xml:space="preserve">Ajoutez ici les moniteurs de la saison : ils apparaîtront automatiquement dans les menus déroulants et dans le récapitulatif. Les mois sont dans l’ordre du calendrier, ne les déplacez pas.</t>
@@ -4527,397 +4581,397 @@
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="21" t="str">
         <f aca="false">IF(Listes!A7="","",Listes!A7)</f>
-        <v/>
-      </c>
-      <c r="B11" s="22" t="str">
+        <v>Thibault</v>
+      </c>
+      <c r="B11" s="22" t="n">
         <f aca="false">IF($A11="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A11,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="C11" s="22" t="str">
+        <v>0</v>
+      </c>
+      <c r="C11" s="22" t="n">
         <f aca="false">IF($A11="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A11,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="D11" s="23" t="str">
+        <v>0</v>
+      </c>
+      <c r="D11" s="23" t="n">
         <f aca="false">IF($A11="","",SUMIF(Remplacements!$E$6:$E$255,$A11,Remplacements!$C$6:$C$255))</f>
-        <v/>
-      </c>
-      <c r="E11" s="23" t="str">
+        <v>0</v>
+      </c>
+      <c r="E11" s="23" t="n">
         <f aca="false">IF($A11="","",SUMIF(Remplacements!$D$6:$D$255,$A11,Remplacements!$C$6:$C$255))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="str">
         <f aca="false">IF(Listes!A8="","",Listes!A8)</f>
-        <v/>
-      </c>
-      <c r="B12" s="19" t="str">
+        <v>Philippe</v>
+      </c>
+      <c r="B12" s="19" t="n">
         <f aca="false">IF($A12="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A12,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="C12" s="19" t="str">
+        <v>0</v>
+      </c>
+      <c r="C12" s="19" t="n">
         <f aca="false">IF($A12="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A12,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="D12" s="20" t="str">
+        <v>0</v>
+      </c>
+      <c r="D12" s="20" t="n">
         <f aca="false">IF($A12="","",SUMIF(Remplacements!$E$6:$E$255,$A12,Remplacements!$C$6:$C$255))</f>
-        <v/>
-      </c>
-      <c r="E12" s="20" t="str">
+        <v>0</v>
+      </c>
+      <c r="E12" s="20" t="n">
         <f aca="false">IF($A12="","",SUMIF(Remplacements!$D$6:$D$255,$A12,Remplacements!$C$6:$C$255))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="21" t="str">
         <f aca="false">IF(Listes!A9="","",Listes!A9)</f>
-        <v/>
-      </c>
-      <c r="B13" s="22" t="str">
+        <v>Adel</v>
+      </c>
+      <c r="B13" s="22" t="n">
         <f aca="false">IF($A13="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A13,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="C13" s="22" t="str">
+        <v>0</v>
+      </c>
+      <c r="C13" s="22" t="n">
         <f aca="false">IF($A13="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A13,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="D13" s="23" t="str">
+        <v>0</v>
+      </c>
+      <c r="D13" s="23" t="n">
         <f aca="false">IF($A13="","",SUMIF(Remplacements!$E$6:$E$255,$A13,Remplacements!$C$6:$C$255))</f>
-        <v/>
-      </c>
-      <c r="E13" s="23" t="str">
+        <v>0</v>
+      </c>
+      <c r="E13" s="23" t="n">
         <f aca="false">IF($A13="","",SUMIF(Remplacements!$D$6:$D$255,$A13,Remplacements!$C$6:$C$255))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="str">
         <f aca="false">IF(Listes!A10="","",Listes!A10)</f>
-        <v/>
-      </c>
-      <c r="B14" s="19" t="str">
+        <v>Alpaslan</v>
+      </c>
+      <c r="B14" s="19" t="n">
         <f aca="false">IF($A14="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A14,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="C14" s="19" t="str">
+        <v>0</v>
+      </c>
+      <c r="C14" s="19" t="n">
         <f aca="false">IF($A14="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A14,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="D14" s="20" t="str">
+        <v>0</v>
+      </c>
+      <c r="D14" s="20" t="n">
         <f aca="false">IF($A14="","",SUMIF(Remplacements!$E$6:$E$255,$A14,Remplacements!$C$6:$C$255))</f>
-        <v/>
-      </c>
-      <c r="E14" s="20" t="str">
+        <v>0</v>
+      </c>
+      <c r="E14" s="20" t="n">
         <f aca="false">IF($A14="","",SUMIF(Remplacements!$D$6:$D$255,$A14,Remplacements!$C$6:$C$255))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="21" t="str">
         <f aca="false">IF(Listes!A11="","",Listes!A11)</f>
-        <v/>
-      </c>
-      <c r="B15" s="22" t="str">
+        <v>Armelle</v>
+      </c>
+      <c r="B15" s="22" t="n">
         <f aca="false">IF($A15="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A15,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="C15" s="22" t="str">
+        <v>0</v>
+      </c>
+      <c r="C15" s="22" t="n">
         <f aca="false">IF($A15="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A15,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="D15" s="23" t="str">
+        <v>0</v>
+      </c>
+      <c r="D15" s="23" t="n">
         <f aca="false">IF($A15="","",SUMIF(Remplacements!$E$6:$E$255,$A15,Remplacements!$C$6:$C$255))</f>
-        <v/>
-      </c>
-      <c r="E15" s="23" t="str">
+        <v>0</v>
+      </c>
+      <c r="E15" s="23" t="n">
         <f aca="false">IF($A15="","",SUMIF(Remplacements!$D$6:$D$255,$A15,Remplacements!$C$6:$C$255))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="str">
         <f aca="false">IF(Listes!A12="","",Listes!A12)</f>
-        <v/>
-      </c>
-      <c r="B16" s="19" t="str">
+        <v>Celia</v>
+      </c>
+      <c r="B16" s="19" t="n">
         <f aca="false">IF($A16="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A16,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="C16" s="19" t="str">
+        <v>0</v>
+      </c>
+      <c r="C16" s="19" t="n">
         <f aca="false">IF($A16="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A16,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="D16" s="20" t="str">
+        <v>0</v>
+      </c>
+      <c r="D16" s="20" t="n">
         <f aca="false">IF($A16="","",SUMIF(Remplacements!$E$6:$E$255,$A16,Remplacements!$C$6:$C$255))</f>
-        <v/>
-      </c>
-      <c r="E16" s="20" t="str">
+        <v>0</v>
+      </c>
+      <c r="E16" s="20" t="n">
         <f aca="false">IF($A16="","",SUMIF(Remplacements!$D$6:$D$255,$A16,Remplacements!$C$6:$C$255))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="21" t="str">
         <f aca="false">IF(Listes!A13="","",Listes!A13)</f>
-        <v/>
-      </c>
-      <c r="B17" s="22" t="str">
+        <v>Clément</v>
+      </c>
+      <c r="B17" s="22" t="n">
         <f aca="false">IF($A17="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A17,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="C17" s="22" t="str">
+        <v>0</v>
+      </c>
+      <c r="C17" s="22" t="n">
         <f aca="false">IF($A17="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A17,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="D17" s="23" t="str">
+        <v>0</v>
+      </c>
+      <c r="D17" s="23" t="n">
         <f aca="false">IF($A17="","",SUMIF(Remplacements!$E$6:$E$255,$A17,Remplacements!$C$6:$C$255))</f>
-        <v/>
-      </c>
-      <c r="E17" s="23" t="str">
+        <v>0</v>
+      </c>
+      <c r="E17" s="23" t="n">
         <f aca="false">IF($A17="","",SUMIF(Remplacements!$D$6:$D$255,$A17,Remplacements!$C$6:$C$255))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="str">
         <f aca="false">IF(Listes!A14="","",Listes!A14)</f>
-        <v/>
-      </c>
-      <c r="B18" s="19" t="str">
+        <v>Fred</v>
+      </c>
+      <c r="B18" s="19" t="n">
         <f aca="false">IF($A18="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A18,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="C18" s="19" t="str">
+        <v>0</v>
+      </c>
+      <c r="C18" s="19" t="n">
         <f aca="false">IF($A18="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A18,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="D18" s="20" t="str">
+        <v>0</v>
+      </c>
+      <c r="D18" s="20" t="n">
         <f aca="false">IF($A18="","",SUMIF(Remplacements!$E$6:$E$255,$A18,Remplacements!$C$6:$C$255))</f>
-        <v/>
-      </c>
-      <c r="E18" s="20" t="str">
+        <v>0</v>
+      </c>
+      <c r="E18" s="20" t="n">
         <f aca="false">IF($A18="","",SUMIF(Remplacements!$D$6:$D$255,$A18,Remplacements!$C$6:$C$255))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="21" t="str">
         <f aca="false">IF(Listes!A15="","",Listes!A15)</f>
-        <v/>
-      </c>
-      <c r="B19" s="22" t="str">
+        <v>Guillaume</v>
+      </c>
+      <c r="B19" s="22" t="n">
         <f aca="false">IF($A19="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A19,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="C19" s="22" t="str">
+        <v>0</v>
+      </c>
+      <c r="C19" s="22" t="n">
         <f aca="false">IF($A19="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A19,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="D19" s="23" t="str">
+        <v>0</v>
+      </c>
+      <c r="D19" s="23" t="n">
         <f aca="false">IF($A19="","",SUMIF(Remplacements!$E$6:$E$255,$A19,Remplacements!$C$6:$C$255))</f>
-        <v/>
-      </c>
-      <c r="E19" s="23" t="str">
+        <v>0</v>
+      </c>
+      <c r="E19" s="23" t="n">
         <f aca="false">IF($A19="","",SUMIF(Remplacements!$D$6:$D$255,$A19,Remplacements!$C$6:$C$255))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="18" t="str">
         <f aca="false">IF(Listes!A16="","",Listes!A16)</f>
-        <v/>
-      </c>
-      <c r="B20" s="19" t="str">
+        <v>Jad</v>
+      </c>
+      <c r="B20" s="19" t="n">
         <f aca="false">IF($A20="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A20,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="C20" s="19" t="str">
+        <v>0</v>
+      </c>
+      <c r="C20" s="19" t="n">
         <f aca="false">IF($A20="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A20,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="D20" s="20" t="str">
+        <v>0</v>
+      </c>
+      <c r="D20" s="20" t="n">
         <f aca="false">IF($A20="","",SUMIF(Remplacements!$E$6:$E$255,$A20,Remplacements!$C$6:$C$255))</f>
-        <v/>
-      </c>
-      <c r="E20" s="20" t="str">
+        <v>0</v>
+      </c>
+      <c r="E20" s="20" t="n">
         <f aca="false">IF($A20="","",SUMIF(Remplacements!$D$6:$D$255,$A20,Remplacements!$C$6:$C$255))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="21" t="str">
         <f aca="false">IF(Listes!A17="","",Listes!A17)</f>
-        <v/>
-      </c>
-      <c r="B21" s="22" t="str">
+        <v>Jérémie</v>
+      </c>
+      <c r="B21" s="22" t="n">
         <f aca="false">IF($A21="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A21,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="C21" s="22" t="str">
+        <v>0</v>
+      </c>
+      <c r="C21" s="22" t="n">
         <f aca="false">IF($A21="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A21,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="D21" s="23" t="str">
+        <v>0</v>
+      </c>
+      <c r="D21" s="23" t="n">
         <f aca="false">IF($A21="","",SUMIF(Remplacements!$E$6:$E$255,$A21,Remplacements!$C$6:$C$255))</f>
-        <v/>
-      </c>
-      <c r="E21" s="23" t="str">
+        <v>0</v>
+      </c>
+      <c r="E21" s="23" t="n">
         <f aca="false">IF($A21="","",SUMIF(Remplacements!$D$6:$D$255,$A21,Remplacements!$C$6:$C$255))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="18" t="str">
         <f aca="false">IF(Listes!A18="","",Listes!A18)</f>
-        <v/>
-      </c>
-      <c r="B22" s="19" t="str">
+        <v>Loïc</v>
+      </c>
+      <c r="B22" s="19" t="n">
         <f aca="false">IF($A22="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A22,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="C22" s="19" t="str">
+        <v>0</v>
+      </c>
+      <c r="C22" s="19" t="n">
         <f aca="false">IF($A22="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A22,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="D22" s="20" t="str">
+        <v>0</v>
+      </c>
+      <c r="D22" s="20" t="n">
         <f aca="false">IF($A22="","",SUMIF(Remplacements!$E$6:$E$255,$A22,Remplacements!$C$6:$C$255))</f>
-        <v/>
-      </c>
-      <c r="E22" s="20" t="str">
+        <v>0</v>
+      </c>
+      <c r="E22" s="20" t="n">
         <f aca="false">IF($A22="","",SUMIF(Remplacements!$D$6:$D$255,$A22,Remplacements!$C$6:$C$255))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="21" t="str">
         <f aca="false">IF(Listes!A19="","",Listes!A19)</f>
-        <v/>
-      </c>
-      <c r="B23" s="22" t="str">
+        <v>Morad</v>
+      </c>
+      <c r="B23" s="22" t="n">
         <f aca="false">IF($A23="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A23,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="C23" s="22" t="str">
+        <v>0</v>
+      </c>
+      <c r="C23" s="22" t="n">
         <f aca="false">IF($A23="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A23,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="D23" s="23" t="str">
+        <v>0</v>
+      </c>
+      <c r="D23" s="23" t="n">
         <f aca="false">IF($A23="","",SUMIF(Remplacements!$E$6:$E$255,$A23,Remplacements!$C$6:$C$255))</f>
-        <v/>
-      </c>
-      <c r="E23" s="23" t="str">
+        <v>0</v>
+      </c>
+      <c r="E23" s="23" t="n">
         <f aca="false">IF($A23="","",SUMIF(Remplacements!$D$6:$D$255,$A23,Remplacements!$C$6:$C$255))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="str">
         <f aca="false">IF(Listes!A20="","",Listes!A20)</f>
-        <v/>
-      </c>
-      <c r="B24" s="19" t="str">
+        <v>Pascal</v>
+      </c>
+      <c r="B24" s="19" t="n">
         <f aca="false">IF($A24="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A24,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="C24" s="19" t="str">
+        <v>0</v>
+      </c>
+      <c r="C24" s="19" t="n">
         <f aca="false">IF($A24="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A24,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="D24" s="20" t="str">
+        <v>0</v>
+      </c>
+      <c r="D24" s="20" t="n">
         <f aca="false">IF($A24="","",SUMIF(Remplacements!$E$6:$E$255,$A24,Remplacements!$C$6:$C$255))</f>
-        <v/>
-      </c>
-      <c r="E24" s="20" t="str">
+        <v>0</v>
+      </c>
+      <c r="E24" s="20" t="n">
         <f aca="false">IF($A24="","",SUMIF(Remplacements!$D$6:$D$255,$A24,Remplacements!$C$6:$C$255))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="21" t="str">
         <f aca="false">IF(Listes!A21="","",Listes!A21)</f>
-        <v/>
-      </c>
-      <c r="B25" s="22" t="str">
+        <v>Thibaut</v>
+      </c>
+      <c r="B25" s="22" t="n">
         <f aca="false">IF($A25="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A25,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="C25" s="22" t="str">
+        <v>0</v>
+      </c>
+      <c r="C25" s="22" t="n">
         <f aca="false">IF($A25="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A25,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="D25" s="23" t="str">
+        <v>0</v>
+      </c>
+      <c r="D25" s="23" t="n">
         <f aca="false">IF($A25="","",SUMIF(Remplacements!$E$6:$E$255,$A25,Remplacements!$C$6:$C$255))</f>
-        <v/>
-      </c>
-      <c r="E25" s="23" t="str">
+        <v>0</v>
+      </c>
+      <c r="E25" s="23" t="n">
         <f aca="false">IF($A25="","",SUMIF(Remplacements!$D$6:$D$255,$A25,Remplacements!$C$6:$C$255))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="18" t="str">
         <f aca="false">IF(Listes!A22="","",Listes!A22)</f>
-        <v/>
-      </c>
-      <c r="B26" s="19" t="str">
+        <v>Xavier</v>
+      </c>
+      <c r="B26" s="19" t="n">
         <f aca="false">IF($A26="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A26,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="C26" s="19" t="str">
+        <v>0</v>
+      </c>
+      <c r="C26" s="19" t="n">
         <f aca="false">IF($A26="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A26,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="D26" s="20" t="str">
+        <v>0</v>
+      </c>
+      <c r="D26" s="20" t="n">
         <f aca="false">IF($A26="","",SUMIF(Remplacements!$E$6:$E$255,$A26,Remplacements!$C$6:$C$255))</f>
-        <v/>
-      </c>
-      <c r="E26" s="20" t="str">
+        <v>0</v>
+      </c>
+      <c r="E26" s="20" t="n">
         <f aca="false">IF($A26="","",SUMIF(Remplacements!$D$6:$D$255,$A26,Remplacements!$C$6:$C$255))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="21" t="str">
         <f aca="false">IF(Listes!A23="","",Listes!A23)</f>
-        <v/>
-      </c>
-      <c r="B27" s="22" t="str">
+        <v>Zeliha</v>
+      </c>
+      <c r="B27" s="22" t="n">
         <f aca="false">IF($A27="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A27,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="C27" s="22" t="str">
+        <v>0</v>
+      </c>
+      <c r="C27" s="22" t="n">
         <f aca="false">IF($A27="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A27,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="D27" s="23" t="str">
+        <v>0</v>
+      </c>
+      <c r="D27" s="23" t="n">
         <f aca="false">IF($A27="","",SUMIF(Remplacements!$E$6:$E$255,$A27,Remplacements!$C$6:$C$255))</f>
-        <v/>
-      </c>
-      <c r="E27" s="23" t="str">
+        <v>0</v>
+      </c>
+      <c r="E27" s="23" t="n">
         <f aca="false">IF($A27="","",SUMIF(Remplacements!$D$6:$D$255,$A27,Remplacements!$C$6:$C$255))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="18" t="str">
         <f aca="false">IF(Listes!A24="","",Listes!A24)</f>
-        <v/>
-      </c>
-      <c r="B28" s="19" t="str">
+        <v>Camelia</v>
+      </c>
+      <c r="B28" s="19" t="n">
         <f aca="false">IF($A28="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$E$6:$E$255,$A28,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="C28" s="19" t="str">
+        <v>0</v>
+      </c>
+      <c r="C28" s="19" t="n">
         <f aca="false">IF($A28="","",SUMIFS(Remplacements!$C$6:$C$255,Remplacements!$D$6:$D$255,$A28,Remplacements!$G$6:$G$255,$B$3))</f>
-        <v/>
-      </c>
-      <c r="D28" s="20" t="str">
+        <v>0</v>
+      </c>
+      <c r="D28" s="20" t="n">
         <f aca="false">IF($A28="","",SUMIF(Remplacements!$E$6:$E$255,$A28,Remplacements!$C$6:$C$255))</f>
-        <v/>
-      </c>
-      <c r="E28" s="20" t="str">
+        <v>0</v>
+      </c>
+      <c r="E28" s="20" t="n">
         <f aca="false">IF($A28="","",SUMIF(Remplacements!$D$6:$D$255,$A28,Remplacements!$C$6:$C$255))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5656,47 +5710,59 @@
       <c r="D6" s="18"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="28"/>
+      <c r="A7" s="28" t="s">
+        <v>59</v>
+      </c>
       <c r="B7" s="18"/>
       <c r="C7" s="18" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D7" s="18"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="28"/>
+      <c r="A8" s="28" t="s">
+        <v>61</v>
+      </c>
       <c r="B8" s="18"/>
       <c r="C8" s="18" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D8" s="18"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="28"/>
+      <c r="A9" s="28" t="s">
+        <v>63</v>
+      </c>
       <c r="B9" s="18"/>
       <c r="C9" s="18" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D9" s="18"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="28"/>
+      <c r="A10" s="28" t="s">
+        <v>65</v>
+      </c>
       <c r="B10" s="18"/>
       <c r="C10" s="18" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="D10" s="18"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="28"/>
+      <c r="A11" s="28" t="s">
+        <v>67</v>
+      </c>
       <c r="B11" s="18"/>
       <c r="C11" s="18" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="D11" s="18"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="28"/>
+      <c r="A12" s="28" t="s">
+        <v>69</v>
+      </c>
       <c r="B12" s="18"/>
       <c r="C12" s="18" t="s">
         <v>30</v>
@@ -5704,75 +5770,99 @@
       <c r="D12" s="18"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="28"/>
+      <c r="A13" s="28" t="s">
+        <v>70</v>
+      </c>
       <c r="B13" s="18"/>
       <c r="C13" s="18" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="D13" s="18"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="28"/>
+      <c r="A14" s="28" t="s">
+        <v>72</v>
+      </c>
       <c r="B14" s="18"/>
       <c r="C14" s="18"/>
       <c r="D14" s="18"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="28"/>
+      <c r="A15" s="28" t="s">
+        <v>73</v>
+      </c>
       <c r="B15" s="18"/>
       <c r="C15" s="18"/>
       <c r="D15" s="18"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="28"/>
+      <c r="A16" s="28" t="s">
+        <v>74</v>
+      </c>
       <c r="B16" s="18"/>
       <c r="C16" s="18"/>
       <c r="D16" s="18"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="28"/>
+      <c r="A17" s="28" t="s">
+        <v>75</v>
+      </c>
       <c r="B17" s="18"/>
       <c r="C17" s="18"/>
       <c r="D17" s="18"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="28"/>
+      <c r="A18" s="28" t="s">
+        <v>76</v>
+      </c>
       <c r="B18" s="18"/>
       <c r="C18" s="18"/>
       <c r="D18" s="18"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="28"/>
+      <c r="A19" s="28" t="s">
+        <v>77</v>
+      </c>
       <c r="B19" s="18"/>
       <c r="C19" s="18"/>
       <c r="D19" s="18"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="28"/>
+      <c r="A20" s="28" t="s">
+        <v>78</v>
+      </c>
       <c r="B20" s="18"/>
       <c r="C20" s="18"/>
       <c r="D20" s="18"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="28"/>
+      <c r="A21" s="28" t="s">
+        <v>79</v>
+      </c>
       <c r="B21" s="18"/>
       <c r="C21" s="18"/>
       <c r="D21" s="18"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="28"/>
+      <c r="A22" s="28" t="s">
+        <v>80</v>
+      </c>
       <c r="B22" s="18"/>
       <c r="C22" s="18"/>
       <c r="D22" s="18"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="28"/>
+      <c r="A23" s="28" t="s">
+        <v>81</v>
+      </c>
       <c r="B23" s="18"/>
       <c r="C23" s="18"/>
       <c r="D23" s="18"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="28"/>
+      <c r="A24" s="28" t="s">
+        <v>82</v>
+      </c>
       <c r="B24" s="18"/>
       <c r="C24" s="18"/>
       <c r="D24" s="18"/>
@@ -5941,7 +6031,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="26" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="B54" s="26"/>
       <c r="C54" s="26"/>

</xml_diff>